<commit_message>
Remove temporary configuration file and update documentation references in Local Monitor Dashboard
This commit deletes the temporary configuration file `~$Konfigurasi.xlsx` and updates the documentation reference in the `Local Monitor Dashboard` Python script to point to the newly created `Ship Auto Way Maps Points Tracking.md`. Additionally, a new setup group is added to the dashboard for improved user interaction, enhancing the overall functionality of the application.
</commit_message>
<xml_diff>
--- a/Dokumentasi/Konfigurasi.xlsx
+++ b/Dokumentasi/Konfigurasi.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\inskal-lab-hidro\Kerjaan_Kantor\Pengujian\Ship_Model_Control_ESP32-S3 v2026\Dokumentasi\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pengujian\Ship_Model_Control_ESP32-S3 v2026.01\Dokumentasi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E58F0356-59C7-4430-A005-5BA18D3B5ECB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B0B0C1B-C9E9-4F07-AC4F-65D71065A682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SN_MacAdress" sheetId="1" r:id="rId1"/>
@@ -918,6 +918,9 @@
     <xf numFmtId="15" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -938,9 +941,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -12494,6 +12494,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Sheet1"/>
@@ -13346,11 +13347,11 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
     </row>
     <row r="3" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
@@ -14297,15 +14298,15 @@
       </c>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B35" s="14" t="s">
+      <c r="B35" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+      <c r="H35" s="15"/>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B36" s="9" t="s">
@@ -14528,10 +14529,10 @@
       <c r="H45" s="11"/>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B47" s="15" t="s">
+      <c r="B47" s="16" t="s">
         <v>161</v>
       </c>
-      <c r="C47" s="15"/>
+      <c r="C47" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -14582,11 +14583,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="17" t="s">
         <v>229</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -14831,10 +14832,10 @@
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="16" t="s">
+      <c r="A25" s="17" t="s">
         <v>144</v>
       </c>
-      <c r="B25" s="16"/>
+      <c r="B25" s="17"/>
       <c r="C25" s="3">
         <f>SUM(C4:C24)</f>
         <v>32</v>
@@ -14879,7 +14880,7 @@
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="18" t="s">
         <v>39</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -14896,7 +14897,7 @@
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B5" s="17"/>
+      <c r="B5" s="18"/>
       <c r="C5" s="2" t="s">
         <v>37</v>
       </c>
@@ -14911,7 +14912,7 @@
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B6" s="17"/>
+      <c r="B6" s="18"/>
       <c r="C6" s="2" t="s">
         <v>38</v>
       </c>
@@ -14926,7 +14927,7 @@
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="17"/>
+      <c r="B7" s="18"/>
       <c r="C7" s="2" t="s">
         <v>41</v>
       </c>
@@ -14941,7 +14942,7 @@
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="18" t="s">
         <v>44</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -14956,7 +14957,7 @@
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="17"/>
+      <c r="B9" s="18"/>
       <c r="C9" s="2" t="s">
         <v>40</v>
       </c>
@@ -14971,7 +14972,7 @@
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="17"/>
+      <c r="B10" s="18"/>
       <c r="C10" s="2" t="s">
         <v>46</v>
       </c>
@@ -14986,7 +14987,7 @@
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="17"/>
+      <c r="B11" s="18"/>
       <c r="C11" s="2" t="s">
         <v>47</v>
       </c>
@@ -14996,12 +14997,12 @@
       <c r="E11" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="19" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B12" s="17"/>
+      <c r="B12" s="18"/>
       <c r="C12" s="2" t="s">
         <v>48</v>
       </c>
@@ -15011,10 +15012,10 @@
       <c r="E12" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F12" s="19"/>
+      <c r="F12" s="20"/>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="18" t="s">
         <v>51</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -15026,12 +15027,12 @@
       <c r="E13" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F13" s="17" t="s">
+      <c r="F13" s="18" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="17"/>
+      <c r="B14" s="18"/>
       <c r="C14" s="2" t="s">
         <v>53</v>
       </c>
@@ -15041,10 +15042,10 @@
       <c r="E14" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F14" s="17"/>
+      <c r="F14" s="18"/>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="17"/>
+      <c r="B15" s="18"/>
       <c r="C15" s="2" t="s">
         <v>40</v>
       </c>
@@ -15059,7 +15060,7 @@
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B16" s="17"/>
+      <c r="B16" s="18"/>
       <c r="C16" s="2" t="s">
         <v>46</v>
       </c>
@@ -15074,7 +15075,7 @@
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="19" t="s">
         <v>108</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -15091,7 +15092,7 @@
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="20"/>
+      <c r="B18" s="21"/>
       <c r="C18" s="2" t="s">
         <v>66</v>
       </c>
@@ -15106,7 +15107,7 @@
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="20"/>
+      <c r="B19" s="21"/>
       <c r="C19" s="2" t="s">
         <v>40</v>
       </c>
@@ -15121,14 +15122,14 @@
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B20" s="20"/>
+      <c r="B20" s="21"/>
       <c r="C20" s="2" t="s">
         <v>96</v>
       </c>
       <c r="D20" s="3">
         <v>9</v>
       </c>
-      <c r="E20" s="18" t="s">
+      <c r="E20" s="19" t="s">
         <v>98</v>
       </c>
       <c r="F20" s="3" t="s">
@@ -15136,20 +15137,20 @@
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="19"/>
+      <c r="B21" s="20"/>
       <c r="C21" s="2" t="s">
         <v>97</v>
       </c>
       <c r="D21" s="3">
         <v>10</v>
       </c>
-      <c r="E21" s="19"/>
+      <c r="E21" s="20"/>
       <c r="F21" s="3" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="18" t="s">
         <v>90</v>
       </c>
       <c r="C22" s="2" t="s">
@@ -15161,12 +15162,12 @@
       <c r="E22" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F22" s="17" t="s">
+      <c r="F22" s="18" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="17"/>
+      <c r="B23" s="18"/>
       <c r="C23" s="2" t="s">
         <v>53</v>
       </c>
@@ -15176,10 +15177,10 @@
       <c r="E23" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F23" s="17"/>
+      <c r="F23" s="18"/>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B24" s="17"/>
+      <c r="B24" s="18"/>
       <c r="C24" s="2" t="s">
         <v>40</v>
       </c>
@@ -15194,7 +15195,7 @@
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B25" s="17"/>
+      <c r="B25" s="18"/>
       <c r="C25" s="2" t="s">
         <v>46</v>
       </c>
@@ -15209,7 +15210,7 @@
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="18" t="s">
         <v>105</v>
       </c>
       <c r="C26" s="2" t="s">
@@ -15226,7 +15227,7 @@
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B27" s="17"/>
+      <c r="B27" s="18"/>
       <c r="C27" s="2" t="s">
         <v>107</v>
       </c>
@@ -15287,7 +15288,7 @@
       </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="18" t="s">
         <v>57</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -15295,37 +15296,37 @@
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B4" s="17"/>
+      <c r="B4" s="18"/>
       <c r="C4" s="2" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B5" s="17"/>
+      <c r="B5" s="18"/>
       <c r="C5" s="2" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B6" s="17"/>
+      <c r="B6" s="18"/>
       <c r="C6" s="2" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B7" s="17"/>
+      <c r="B7" s="18"/>
       <c r="C7" s="2" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B8" s="17"/>
+      <c r="B8" s="18"/>
       <c r="C8" s="2" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B9" s="17"/>
+      <c r="B9" s="18"/>
       <c r="C9" s="2" t="s">
         <v>64</v>
       </c>
@@ -15406,28 +15407,28 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21" t="s">
+      <c r="C3" s="14"/>
+      <c r="D3" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="E3" s="21"/>
+      <c r="E3" s="14"/>
       <c r="F3" s="1" t="s">
         <v>33</v>
       </c>
@@ -15961,28 +15962,28 @@
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="21"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="21"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B22" s="21" t="s">
+      <c r="B22" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="21"/>
-      <c r="D22" s="21" t="s">
+      <c r="C22" s="14"/>
+      <c r="D22" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="E22" s="21"/>
+      <c r="E22" s="14"/>
       <c r="F22" s="1" t="s">
         <v>33</v>
       </c>
@@ -16541,11 +16542,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
@@ -17098,48 +17099,48 @@
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="17"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="18"/>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="18" t="s">
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="16" t="s">
+      <c r="F8" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
-      <c r="I8" s="17" t="s">
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="18"/>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="19"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="20"/>
       <c r="F9" s="2" t="s">
         <v>20</v>
       </c>
@@ -17160,7 +17161,7 @@
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B10" s="17"/>
+      <c r="B10" s="18"/>
       <c r="C10" s="3" t="s">
         <v>12</v>
       </c>
@@ -17190,7 +17191,7 @@
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B11" s="17"/>
+      <c r="B11" s="18"/>
       <c r="C11" s="3" t="s">
         <v>13</v>
       </c>
@@ -17220,7 +17221,7 @@
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B12" s="17"/>
+      <c r="B12" s="18"/>
       <c r="C12" s="3" t="s">
         <v>14</v>
       </c>
@@ -17250,7 +17251,7 @@
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B13" s="17"/>
+      <c r="B13" s="18"/>
       <c r="C13" s="3" t="s">
         <v>15</v>
       </c>

</xml_diff>

<commit_message>
Update PlatformIO configuration and add new Excel file
This commit updates the `platformio.ini` files for two ESP-NOW projects, changing the upload and monitor ports to ensure proper communication. Additionally, a new temporary Excel file `~$Konfigurasi.xlsx` has been added to the documentation directory. These changes enhance the project setup and facilitate smoother development processes.
</commit_message>
<xml_diff>
--- a/Dokumentasi/Konfigurasi.xlsx
+++ b/Dokumentasi/Konfigurasi.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pengujian\Ship_Model_Control_ESP32-S3 v2026.01\Dokumentasi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B0B0C1B-C9E9-4F07-AC4F-65D71065A682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0CED2AF-6BD7-4ACD-BA34-583D97AB4AFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="244">
   <si>
     <t>Transmitter</t>
   </si>
@@ -765,6 +765,12 @@
   </si>
   <si>
     <t>intercept</t>
+  </si>
+  <si>
+    <t>ESP32-S3 Sender</t>
+  </si>
+  <si>
+    <t>98:a3:16:f5:01:a0</t>
   </si>
 </sst>
 </file>
@@ -881,7 +887,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -918,9 +924,6 @@
     <xf numFmtId="15" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -942,12 +945,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -12887,7 +12897,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:D9"/>
+  <dimension ref="B2:D10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="28.6640625" bestFit="1" customWidth="1"/>
@@ -12958,6 +12968,14 @@
       </c>
       <c r="C9" s="3" t="s">
         <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B10" s="24" t="s">
+        <v>242</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -13347,11 +13365,11 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
     </row>
     <row r="3" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
@@ -14298,15 +14316,15 @@
       </c>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B35" s="15" t="s">
+      <c r="B35" s="14" t="s">
         <v>151</v>
       </c>
-      <c r="C35" s="15"/>
-      <c r="D35" s="15"/>
-      <c r="E35" s="15"/>
-      <c r="F35" s="15"/>
-      <c r="G35" s="15"/>
-      <c r="H35" s="15"/>
+      <c r="C35" s="14"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="14"/>
+      <c r="G35" s="14"/>
+      <c r="H35" s="14"/>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B36" s="9" t="s">
@@ -14529,10 +14547,10 @@
       <c r="H45" s="11"/>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B47" s="16" t="s">
+      <c r="B47" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="C47" s="16"/>
+      <c r="C47" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -14583,11 +14601,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="16" t="s">
         <v>229</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -14832,10 +14850,10 @@
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="17" t="s">
+      <c r="A25" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="B25" s="17"/>
+      <c r="B25" s="16"/>
       <c r="C25" s="3">
         <f>SUM(C4:C24)</f>
         <v>32</v>
@@ -14880,7 +14898,7 @@
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="17" t="s">
         <v>39</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -14897,7 +14915,7 @@
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B5" s="18"/>
+      <c r="B5" s="17"/>
       <c r="C5" s="2" t="s">
         <v>37</v>
       </c>
@@ -14912,7 +14930,7 @@
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B6" s="18"/>
+      <c r="B6" s="17"/>
       <c r="C6" s="2" t="s">
         <v>38</v>
       </c>
@@ -14927,7 +14945,7 @@
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="18"/>
+      <c r="B7" s="17"/>
       <c r="C7" s="2" t="s">
         <v>41</v>
       </c>
@@ -14942,7 +14960,7 @@
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="17" t="s">
         <v>44</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -14957,7 +14975,7 @@
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="18"/>
+      <c r="B9" s="17"/>
       <c r="C9" s="2" t="s">
         <v>40</v>
       </c>
@@ -14972,7 +14990,7 @@
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="18"/>
+      <c r="B10" s="17"/>
       <c r="C10" s="2" t="s">
         <v>46</v>
       </c>
@@ -14987,7 +15005,7 @@
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="18"/>
+      <c r="B11" s="17"/>
       <c r="C11" s="2" t="s">
         <v>47</v>
       </c>
@@ -14997,12 +15015,12 @@
       <c r="E11" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="19" t="s">
+      <c r="F11" s="18" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B12" s="18"/>
+      <c r="B12" s="17"/>
       <c r="C12" s="2" t="s">
         <v>48</v>
       </c>
@@ -15012,10 +15030,10 @@
       <c r="E12" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F12" s="20"/>
+      <c r="F12" s="19"/>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="17" t="s">
         <v>51</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -15027,12 +15045,12 @@
       <c r="E13" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F13" s="18" t="s">
+      <c r="F13" s="17" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="18"/>
+      <c r="B14" s="17"/>
       <c r="C14" s="2" t="s">
         <v>53</v>
       </c>
@@ -15042,10 +15060,10 @@
       <c r="E14" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F14" s="18"/>
+      <c r="F14" s="17"/>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="18"/>
+      <c r="B15" s="17"/>
       <c r="C15" s="2" t="s">
         <v>40</v>
       </c>
@@ -15060,7 +15078,7 @@
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B16" s="18"/>
+      <c r="B16" s="17"/>
       <c r="C16" s="2" t="s">
         <v>46</v>
       </c>
@@ -15075,7 +15093,7 @@
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="18" t="s">
         <v>108</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -15092,7 +15110,7 @@
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="21"/>
+      <c r="B18" s="20"/>
       <c r="C18" s="2" t="s">
         <v>66</v>
       </c>
@@ -15107,7 +15125,7 @@
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="21"/>
+      <c r="B19" s="20"/>
       <c r="C19" s="2" t="s">
         <v>40</v>
       </c>
@@ -15122,14 +15140,14 @@
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B20" s="21"/>
+      <c r="B20" s="20"/>
       <c r="C20" s="2" t="s">
         <v>96</v>
       </c>
       <c r="D20" s="3">
         <v>9</v>
       </c>
-      <c r="E20" s="19" t="s">
+      <c r="E20" s="18" t="s">
         <v>98</v>
       </c>
       <c r="F20" s="3" t="s">
@@ -15137,20 +15155,20 @@
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="20"/>
+      <c r="B21" s="19"/>
       <c r="C21" s="2" t="s">
         <v>97</v>
       </c>
       <c r="D21" s="3">
         <v>10</v>
       </c>
-      <c r="E21" s="20"/>
+      <c r="E21" s="19"/>
       <c r="F21" s="3" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="18" t="s">
+      <c r="B22" s="17" t="s">
         <v>90</v>
       </c>
       <c r="C22" s="2" t="s">
@@ -15162,12 +15180,12 @@
       <c r="E22" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F22" s="18" t="s">
+      <c r="F22" s="17" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="18"/>
+      <c r="B23" s="17"/>
       <c r="C23" s="2" t="s">
         <v>53</v>
       </c>
@@ -15177,10 +15195,10 @@
       <c r="E23" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F23" s="18"/>
+      <c r="F23" s="17"/>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B24" s="18"/>
+      <c r="B24" s="17"/>
       <c r="C24" s="2" t="s">
         <v>40</v>
       </c>
@@ -15195,7 +15213,7 @@
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B25" s="18"/>
+      <c r="B25" s="17"/>
       <c r="C25" s="2" t="s">
         <v>46</v>
       </c>
@@ -15210,7 +15228,7 @@
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B26" s="18" t="s">
+      <c r="B26" s="17" t="s">
         <v>105</v>
       </c>
       <c r="C26" s="2" t="s">
@@ -15227,7 +15245,7 @@
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B27" s="18"/>
+      <c r="B27" s="17"/>
       <c r="C27" s="2" t="s">
         <v>107</v>
       </c>
@@ -15288,7 +15306,7 @@
       </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="17" t="s">
         <v>57</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -15296,37 +15314,37 @@
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B4" s="18"/>
+      <c r="B4" s="17"/>
       <c r="C4" s="2" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B5" s="18"/>
+      <c r="B5" s="17"/>
       <c r="C5" s="2" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B6" s="18"/>
+      <c r="B6" s="17"/>
       <c r="C6" s="2" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B7" s="18"/>
+      <c r="B7" s="17"/>
       <c r="C7" s="2" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B8" s="18"/>
+      <c r="B8" s="17"/>
       <c r="C8" s="2" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B9" s="18"/>
+      <c r="B9" s="17"/>
       <c r="C9" s="2" t="s">
         <v>64</v>
       </c>
@@ -15407,28 +15425,28 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14" t="s">
+      <c r="C3" s="21"/>
+      <c r="D3" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="E3" s="14"/>
+      <c r="E3" s="21"/>
       <c r="F3" s="1" t="s">
         <v>33</v>
       </c>
@@ -15962,28 +15980,28 @@
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="21"/>
+      <c r="D21" s="21"/>
+      <c r="E21" s="21"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="21"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="B22" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14" t="s">
+      <c r="C22" s="21"/>
+      <c r="D22" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="E22" s="14"/>
+      <c r="E22" s="21"/>
       <c r="F22" s="1" t="s">
         <v>33</v>
       </c>
@@ -16542,11 +16560,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
@@ -17099,48 +17117,48 @@
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="18"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="18"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="17"/>
+      <c r="K7" s="17"/>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="19" t="s">
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="17" t="s">
+      <c r="F8" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="18" t="s">
+      <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="J8" s="18"/>
-      <c r="K8" s="18"/>
+      <c r="J8" s="17"/>
+      <c r="K8" s="17"/>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B9" s="18"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="20"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="19"/>
       <c r="F9" s="2" t="s">
         <v>20</v>
       </c>
@@ -17161,7 +17179,7 @@
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B10" s="18"/>
+      <c r="B10" s="17"/>
       <c r="C10" s="3" t="s">
         <v>12</v>
       </c>
@@ -17191,7 +17209,7 @@
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B11" s="18"/>
+      <c r="B11" s="17"/>
       <c r="C11" s="3" t="s">
         <v>13</v>
       </c>
@@ -17221,7 +17239,7 @@
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B12" s="18"/>
+      <c r="B12" s="17"/>
       <c r="C12" s="3" t="s">
         <v>14</v>
       </c>
@@ -17251,7 +17269,7 @@
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B13" s="18"/>
+      <c r="B13" s="17"/>
       <c r="C13" s="3" t="s">
         <v>15</v>
       </c>

</xml_diff>